<commit_message>
terrafrom moduleand added .gitignore
</commit_message>
<xml_diff>
--- a/P-M/Enterprise_Project_Planner_v4.xlsx
+++ b/P-M/Enterprise_Project_Planner_v4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\Desktop\Workspace\Multi-Cloud-Kubernetes-Auto-Healing-Auto-Scaling-Platform\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\Desktop\Workspace\Multi-Cloud-Kubernetes-Auto-Healing-Auto-Scaling-Platform\P-M\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF28171-F59F-4D99-86E2-BDB4F0BEC26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498E4B62-43C1-4911-847E-2922356CF8C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="118">
   <si>
     <t>Metric</t>
   </si>
@@ -360,6 +360,27 @@
   </si>
   <si>
     <t>Terraform, AWS EKS, Azure AKS, IAM, Networking, Git</t>
+  </si>
+  <si>
+    <t xml:space="preserve">folder strutre was create </t>
+  </si>
+  <si>
+    <t>terraform/modules/networking/vnet</t>
+  </si>
+  <si>
+    <t>terraform/modules/eks</t>
+  </si>
+  <si>
+    <t>terraform/modules/aks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">terraform/modules/networking/vpc </t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>End Date</t>
   </si>
 </sst>
 </file>
@@ -409,7 +430,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -419,6 +440,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -428,7 +450,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF00B050"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -442,21 +478,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -929,17 +951,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.77734375" customWidth="1"/>
-    <col min="7" max="7" width="79.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" customWidth="1"/>
+    <col min="5" max="5" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" customWidth="1"/>
+    <col min="9" max="9" width="79.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -947,611 +971,656 @@
         <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="5">
+        <v>46176</v>
+      </c>
+      <c r="D2" s="5">
+        <v>46176</v>
+      </c>
+      <c r="E2" t="s">
         <v>35</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>36</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>4</v>
       </c>
-      <c r="F2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="5">
+        <v>46176</v>
+      </c>
+      <c r="D3" s="5">
+        <v>46176</v>
+      </c>
+      <c r="E3" t="s">
         <v>37</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>38</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>6</v>
       </c>
-      <c r="F3" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" t="s">
+        <v>105</v>
+      </c>
+      <c r="I3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="5">
+        <v>46176</v>
+      </c>
+      <c r="E4" t="s">
         <v>39</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>40</v>
       </c>
-      <c r="E4">
+      <c r="G4">
         <v>6</v>
       </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" t="s">
+        <v>106</v>
+      </c>
+      <c r="I4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="5">
+        <v>46176</v>
+      </c>
+      <c r="E5" t="s">
         <v>41</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>42</v>
       </c>
-      <c r="E5">
+      <c r="G5">
         <v>8</v>
       </c>
-      <c r="F5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" t="s">
+        <v>106</v>
+      </c>
+      <c r="I5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="5">
+        <v>46176</v>
+      </c>
+      <c r="E6" t="s">
         <v>43</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>44</v>
       </c>
-      <c r="E6">
+      <c r="G6">
         <v>6</v>
       </c>
-      <c r="F6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6" t="s">
+        <v>106</v>
+      </c>
+      <c r="I6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>18</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="5">
+        <v>46176</v>
+      </c>
+      <c r="E7" t="s">
         <v>45</v>
       </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>42</v>
       </c>
-      <c r="E7">
+      <c r="G7">
         <v>8</v>
       </c>
-      <c r="F7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>106</v>
+      </c>
+      <c r="I7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>18</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
         <v>46</v>
       </c>
-      <c r="D8" t="s">
+      <c r="F8" t="s">
         <v>47</v>
       </c>
-      <c r="E8">
+      <c r="G8">
         <v>4</v>
       </c>
-      <c r="F8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
+      <c r="E9" t="s">
         <v>48</v>
       </c>
-      <c r="D9" t="s">
+      <c r="F9" t="s">
         <v>49</v>
       </c>
-      <c r="E9">
+      <c r="G9">
         <v>6</v>
       </c>
-      <c r="F9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E10" t="s">
         <v>50</v>
       </c>
-      <c r="D10" t="s">
+      <c r="F10" t="s">
         <v>49</v>
       </c>
-      <c r="E10">
+      <c r="G10">
         <v>6</v>
       </c>
-      <c r="F10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
       </c>
-      <c r="C11" t="s">
+      <c r="E11" t="s">
         <v>51</v>
       </c>
-      <c r="D11" t="s">
+      <c r="F11" t="s">
         <v>52</v>
       </c>
-      <c r="E11">
+      <c r="G11">
         <v>6</v>
       </c>
-      <c r="F11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
         <v>21</v>
       </c>
-      <c r="C12" t="s">
+      <c r="E12" t="s">
         <v>53</v>
       </c>
-      <c r="D12" t="s">
+      <c r="F12" t="s">
         <v>54</v>
       </c>
-      <c r="E12">
+      <c r="G12">
         <v>6</v>
       </c>
-      <c r="F12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
         <v>21</v>
       </c>
-      <c r="C13" t="s">
+      <c r="E13" t="s">
         <v>55</v>
       </c>
-      <c r="D13" t="s">
+      <c r="F13" t="s">
         <v>56</v>
       </c>
-      <c r="E13">
+      <c r="G13">
         <v>6</v>
       </c>
-      <c r="F13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
         <v>21</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" t="s">
         <v>57</v>
       </c>
-      <c r="D14" t="s">
+      <c r="F14" t="s">
         <v>58</v>
       </c>
-      <c r="E14">
+      <c r="G14">
         <v>6</v>
       </c>
-      <c r="F14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
         <v>24</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
         <v>59</v>
       </c>
-      <c r="D15" t="s">
+      <c r="F15" t="s">
         <v>60</v>
       </c>
-      <c r="E15">
+      <c r="G15">
         <v>4</v>
       </c>
-      <c r="F15" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>24</v>
       </c>
-      <c r="C16" t="s">
+      <c r="E16" t="s">
         <v>61</v>
       </c>
-      <c r="D16" t="s">
+      <c r="F16" t="s">
         <v>62</v>
       </c>
-      <c r="E16">
+      <c r="G16">
         <v>4</v>
       </c>
-      <c r="F16" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
         <v>24</v>
       </c>
-      <c r="C17" t="s">
+      <c r="E17" t="s">
         <v>63</v>
       </c>
-      <c r="D17" t="s">
+      <c r="F17" t="s">
         <v>64</v>
       </c>
-      <c r="E17">
+      <c r="G17">
         <v>4</v>
       </c>
-      <c r="F17" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
         <v>24</v>
       </c>
-      <c r="C18" t="s">
+      <c r="E18" t="s">
         <v>65</v>
       </c>
-      <c r="D18" t="s">
+      <c r="F18" t="s">
         <v>66</v>
       </c>
-      <c r="E18">
+      <c r="G18">
         <v>6</v>
       </c>
-      <c r="F18" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H18" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>24</v>
       </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
         <v>67</v>
       </c>
-      <c r="D19" t="s">
+      <c r="F19" t="s">
         <v>68</v>
       </c>
-      <c r="E19">
+      <c r="G19">
         <v>6</v>
       </c>
-      <c r="F19" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
       </c>
-      <c r="C20" t="s">
+      <c r="E20" t="s">
         <v>69</v>
       </c>
-      <c r="D20" t="s">
+      <c r="F20" t="s">
         <v>70</v>
       </c>
-      <c r="E20">
+      <c r="G20">
         <v>4</v>
       </c>
-      <c r="F20" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
         <v>27</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>71</v>
       </c>
-      <c r="D21" t="s">
+      <c r="F21" t="s">
         <v>72</v>
       </c>
-      <c r="E21">
+      <c r="G21">
         <v>4</v>
       </c>
-      <c r="F21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
         <v>27</v>
       </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
         <v>73</v>
       </c>
-      <c r="D22" t="s">
+      <c r="F22" t="s">
         <v>74</v>
       </c>
-      <c r="E22">
+      <c r="G22">
         <v>4</v>
       </c>
-      <c r="F22" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>27</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>75</v>
       </c>
-      <c r="D23" t="s">
+      <c r="F23" t="s">
         <v>76</v>
       </c>
-      <c r="E23">
+      <c r="G23">
         <v>4</v>
       </c>
-      <c r="F23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
         <v>27</v>
       </c>
-      <c r="C24" t="s">
+      <c r="E24" t="s">
         <v>77</v>
       </c>
-      <c r="D24" t="s">
+      <c r="F24" t="s">
         <v>78</v>
       </c>
-      <c r="E24">
+      <c r="G24">
         <v>3</v>
       </c>
-      <c r="F24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H24" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
         <v>27</v>
       </c>
-      <c r="C25" t="s">
+      <c r="E25" t="s">
         <v>79</v>
       </c>
-      <c r="D25" t="s">
+      <c r="F25" t="s">
         <v>80</v>
       </c>
-      <c r="E25">
+      <c r="G25">
         <v>3</v>
       </c>
-      <c r="F25" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H25" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
         <v>27</v>
       </c>
-      <c r="C26" t="s">
+      <c r="E26" t="s">
         <v>81</v>
       </c>
-      <c r="D26" t="s">
+      <c r="F26" t="s">
         <v>82</v>
       </c>
-      <c r="E26">
+      <c r="G26">
         <v>6</v>
       </c>
-      <c r="F26" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H26" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
         <v>27</v>
       </c>
-      <c r="C27" t="s">
+      <c r="E27" t="s">
         <v>83</v>
       </c>
-      <c r="D27" t="s">
+      <c r="F27" t="s">
         <v>84</v>
       </c>
-      <c r="E27">
+      <c r="G27">
         <v>6</v>
       </c>
-      <c r="F27" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
         <v>27</v>
       </c>
-      <c r="C28" t="s">
+      <c r="E28" t="s">
         <v>85</v>
       </c>
-      <c r="D28" t="s">
+      <c r="F28" t="s">
         <v>86</v>
       </c>
-      <c r="E28">
+      <c r="G28">
         <v>2</v>
       </c>
-      <c r="F28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H28" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
         <v>27</v>
       </c>
-      <c r="C29" t="s">
+      <c r="E29" t="s">
         <v>87</v>
       </c>
-      <c r="D29" t="s">
+      <c r="F29" t="s">
         <v>88</v>
       </c>
-      <c r="E29">
+      <c r="G29">
         <v>2</v>
       </c>
-      <c r="F29" t="s">
+      <c r="H29" t="s">
         <v>20</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:G2">
-    <cfRule type="cellIs" dxfId="4" priority="5" stopIfTrue="1" operator="equal">
-      <formula>"Deferred"</formula>
+  <conditionalFormatting sqref="H1:H1048576 I2:I7">
+    <cfRule type="cellIs" dxfId="4" priority="1" stopIfTrue="1" operator="equal">
+      <formula>"Completed"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F1:F1048576 G2">
-    <cfRule type="cellIs" dxfId="3" priority="4" stopIfTrue="1" operator="equal">
-      <formula>"Not Started"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="2" stopIfTrue="1" operator="equal">
+      <formula>"In Progress"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="2" priority="3" stopIfTrue="1" operator="equal">
       <formula>"Blocked "</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="equal">
-      <formula>"In Progress"</formula>
+    <cfRule type="cellIs" dxfId="1" priority="4" stopIfTrue="1" operator="equal">
+      <formula>"Not Started"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">
-      <formula>"Completed"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:I2">
+    <cfRule type="cellIs" dxfId="0" priority="5" stopIfTrue="1" operator="equal">
+      <formula>"Deferred"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F28" xr:uid="{88B4A230-DCAB-4671-9F6F-5A60A415E615}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H28" xr:uid="{88B4A230-DCAB-4671-9F6F-5A60A415E615}">
       <formula1>"Not Started,In Progress,Blocked,Completed,Deferred"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{5F8FFB7B-27E4-4774-B0E8-E6D38E1B73D6}"/>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{5F8FFB7B-27E4-4774-B0E8-E6D38E1B73D6}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>